<commit_message>
Cahier de recette: 2 fiches ciblees sur les points sensibles (CR-22, CR-23)
CR-22: annulation d'une vente ordonnancee/tiers-payant -> valide que le trigger
V6.3.2 solde le differe sans casser la contre-passation tiers-payant.
CR-23: cloture d'une vente depot differee -> valide que la garde d'idempotence
ne bloque pas la creation legitime du differe (chemin addDiffere @2948).
Total recette porte a 23 fiches.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrJky83P5sReR7DTCBPfmY
</commit_message>
<xml_diff>
--- a/scripts/cahier_recette_differes.xlsx
+++ b/scripts/cahier_recette_differes.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Cahier de recette'!$8:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cahier de recette'!$A$1:$F$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cahier de recette'!$A$1:$F$56</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Mise en production'!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1275,77 +1275,101 @@
       <c r="E36" s="10" t="inlineStr"/>
       <c r="F36" s="11" t="inlineStr"/>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="37" ht="88.85714285714286" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>CR-22</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Annulation d'une vente ORDONNANCÉE / tiers-payant (point sensible : trigger V6.3.2)</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>1. Faire une vente ordonnancée / avec tiers-payant, la clôturer.
+2. L'annuler.
+3. Vérifier la comptabilité tiers-payant (part organisme) ET la dette différée du client.</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>La part tiers-payant reste correctement contre-passée (inchangée par rapport à avant). La dette différée du client de la vente annulée est soldée (reste 0, statut delete). Aucun écart comptable nouveau introduit par le trigger.</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr"/>
+      <c r="F37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38" ht="68.28571428571429" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>CR-23</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Clôture d'une vente DÉPÔT différée (point sensible : garde d'idempotence)</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>1. Faire une vente de type dépôt / extension réglée en différé.
+2. La clôturer.
+3. Requête : nb de lignes de différé de la vente.</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>La dette différée est bien créée (exactement UNE ligne active). La garde d'idempotence ne bloque pas la création légitime sur ce chemin (addDiffere @2948).</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr"/>
+      <c r="F38" s="11" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>SYNTHÈSE ET DÉCISION</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Rubrique</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Nb fiches</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>KO</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Réserves</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>A. Règlement sélectif</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="C40" s="15" t="n"/>
-      <c r="D40" s="15" t="n"/>
-      <c r="E40" s="15" t="n"/>
-      <c r="F40" s="15" t="n"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>B. Règlement global</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15" t="n"/>
+      <c r="F41" s="6" t="inlineStr"/>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>C. Annulation</t>
+          <t>A. Règlement sélectif</t>
         </is>
       </c>
       <c r="B42" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C42" s="15" t="n"/>
       <c r="D42" s="15" t="n"/>
@@ -1355,11 +1379,11 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>D. Cohérence des soldes</t>
+          <t>B. Règlement global</t>
         </is>
       </c>
       <c r="B43" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C43" s="15" t="n"/>
       <c r="D43" s="15" t="n"/>
@@ -1369,7 +1393,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>E. Onglet Différés réglés</t>
+          <t>C. Annulation</t>
         </is>
       </c>
       <c r="B44" s="15" t="n">
@@ -1383,11 +1407,11 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>F. Réparation des données</t>
+          <t>D. Cohérence des soldes</t>
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C45" s="15" t="n"/>
       <c r="D45" s="15" t="n"/>
@@ -1397,11 +1421,11 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>G. Non-régression</t>
+          <t>E. Onglet Différés réglés</t>
         </is>
       </c>
       <c r="B46" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C46" s="15" t="n"/>
       <c r="D46" s="15" t="n"/>
@@ -1409,48 +1433,60 @@
       <c r="F46" s="15" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>F. Réparation des données</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15" t="n"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>G. Non-régression</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="15" t="n"/>
+      <c r="F48" s="15" t="n"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B47" s="17" t="n">
-        <v>21</v>
-      </c>
-      <c r="C47" s="17" t="n"/>
-      <c r="D47" s="17" t="n"/>
-      <c r="E47" s="17" t="n"/>
-      <c r="F47" s="17" t="n"/>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="18" t="inlineStr">
+      <c r="B49" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="C49" s="17" t="n"/>
+      <c r="D49" s="17" t="n"/>
+      <c r="E49" s="17" t="n"/>
+      <c r="F49" s="17" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>Décision :   ☐ Recette prononcée sans réserve   •   ☐ Prononcée avec réserves   •   ☐ Refusée</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="19" t="inlineStr">
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>Réserves / observations :</t>
         </is>
       </c>
-      <c r="B50" s="8" t="n"/>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="8" t="n"/>
-      <c r="F50" s="8" t="n"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="20" t="inlineStr"/>
-      <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="8" t="n"/>
-      <c r="E51" s="8" t="n"/>
-      <c r="F51" s="8" t="n"/>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="20" t="inlineStr"/>
       <c r="B52" s="8" t="n"/>
       <c r="C52" s="8" t="n"/>
       <c r="D52" s="8" t="n"/>
@@ -1458,14 +1494,30 @@
       <c r="F52" s="8" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="21" t="inlineStr">
+      <c r="A53" s="20" t="inlineStr"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="n"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="20" t="inlineStr"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="8" t="n"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="21" t="inlineStr">
         <is>
           <t>Testeur : __________________   Date : __________   Signature : __________________</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="21" t="inlineStr">
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="21" t="inlineStr">
         <is>
           <t>Responsable officine : __________________   Date : __________   Signature : __________________</t>
         </is>
@@ -1476,18 +1528,18 @@
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="E5:F5"/>
-    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A55:F55"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A52:F52"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A51:F51"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>